<commit_message>
Feat: Ingesta, pipeline ETL, análisis K-Means y SAT optimizado con galería de gráficos completa
</commit_message>
<xml_diff>
--- a/Docs/Cohortes_OULAD.xlsx
+++ b/Docs/Cohortes_OULAD.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jcabral\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jcabral\Downloads\OULAD\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{EB588E39-305E-4C52-819C-0689B6D4DACD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76E5961C-1DB4-4EB8-9A83-59FEDA760973}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{057E2E03-633E-438A-9ABD-EAE077E8E8C4}"/>
   </bookViews>
@@ -93,13 +93,19 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -238,33 +244,144 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="8">
+  <dxfs count="9">
     <dxf>
-      <border diagonalUp="0" diagonalDown="0">
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
         <right style="thin">
           <color indexed="64"/>
         </right>
-        <top/>
-        <bottom/>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
       </border>
     </dxf>
     <dxf>
@@ -272,90 +389,15 @@
         <left style="thin">
           <color indexed="64"/>
         </left>
-        <right/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
         <top style="thin">
           <color indexed="64"/>
         </top>
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left/>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
       </border>
     </dxf>
     <dxf>
@@ -373,12 +415,14 @@
         <right style="thin">
           <color indexed="64"/>
         </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
+        <top/>
+        <bottom/>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
       </border>
     </dxf>
   </dxfs>
@@ -395,7 +439,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4D7DC100-5A01-4F4A-B9EE-3CB6C14E5CCE}" name="Table1" displayName="Table1" ref="A1:D4" totalsRowShown="0" headerRowDxfId="0" headerRowBorderDxfId="6" tableBorderDxfId="7" totalsRowBorderDxfId="5">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4D7DC100-5A01-4F4A-B9EE-3CB6C14E5CCE}" name="Table1" displayName="Table1" ref="A1:D4" totalsRowShown="0" headerRowDxfId="8" dataDxfId="0" headerRowBorderDxfId="7" tableBorderDxfId="6" totalsRowBorderDxfId="5">
   <autoFilter ref="A1:D4" xr:uid="{4D7DC100-5A01-4F4A-B9EE-3CB6C14E5CCE}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{1B75352A-225A-4C7A-899D-FFB8A8380395}" name="Cohorte de la Tesis" dataDxfId="4"/>
@@ -747,7 +791,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
         <v>4</v>
       </c>
@@ -761,7 +805,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
         <v>8</v>
       </c>
@@ -775,7 +819,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
         <v>12</v>
       </c>

</xml_diff>